<commit_message>
Use real dimension values in validation fixtures
</commit_message>
<xml_diff>
--- a/examples/validation_fixtures/candidate.xlsx
+++ b/examples/validation_fixtures/candidate.xlsx
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INN001</t>
+          <t>APR3F_06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -595,12 +595,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>AddCtrl</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INN001</t>
+          <t>APR3F_06</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>AddCtrl</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -652,7 +652,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INN002</t>
+          <t>APR3G_11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>1980 APR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INN003</t>
+          <t>B0407HP_NRP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -734,7 +734,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INN004</t>
+          <t>B0407HP_RP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -750,12 +750,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>WATER</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -790,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -803,14 +803,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INN001</t>
+          <t>APR3F_06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INN002</t>
+          <t>APR3G_11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B0407HP_NRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B0407HP_RP</t>
         </is>
       </c>
     </row>

</xml_diff>